<commit_message>
refactor: change de URL base for each ATC
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\eclipse-workspace\automation-framework-back\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93AC3D5-C6F8-49EE-A48B-82B8332ECA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E01E2C-C0C0-4541-8845-5004FC7E4E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,40 +165,40 @@
     <t>CORREO@PRUEBA.COM</t>
   </si>
   <si>
+    <t>ATC01_Test1</t>
+  </si>
+  <si>
+    <t>ATC02_Test2</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Id_2</t>
+  </si>
+  <si>
+    <t>9999</t>
+  </si>
+  <si>
+    <t>UserId</t>
+  </si>
+  <si>
+    <t>Schema</t>
+  </si>
+  <si>
+    <t>post-schema</t>
+  </si>
+  <si>
     <t>Ejecutar</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
     <t>SI</t>
-  </si>
-  <si>
-    <t>ATC01_Test1</t>
-  </si>
-  <si>
-    <t>ATC02_Test2</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Id_2</t>
-  </si>
-  <si>
-    <t>9999</t>
-  </si>
-  <si>
-    <t>UserId</t>
-  </si>
-  <si>
-    <t>Schema</t>
-  </si>
-  <si>
-    <t>post-schema</t>
   </si>
 </sst>
 </file>
@@ -272,13 +272,13 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -297,20 +297,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:P4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TestCaseName"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tester"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Version"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Descripcion"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Pais"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Subsidiaria"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Categoria"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="FechaInicial"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="0"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="NombrePersona"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="CargoPersona"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="InternoExterno"/>
@@ -322,11 +322,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:F3" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:F3" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
-    <tableColumn id="5" xr3:uid="{F1AC137C-52ED-4BA8-975F-2B472EF9FAAE}" name="Ejecutar"/>
+    <tableColumn id="5" xr3:uid="{6BE7C047-30A3-421D-870C-CBBC4443BB44}" name="Ejecutar"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="UserId"/>
     <tableColumn id="3" xr3:uid="{2E8C600E-A409-4D88-8FD4-9D0C9284F1EF}" name="Id_2"/>
@@ -843,11 +843,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
@@ -858,47 +859,47 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" t="s">
         <v>50</v>
-      </c>
-      <c r="F2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>52</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -907,7 +908,10 @@
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D7" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D8" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
feat: New login functionality added
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\eclipse-workspace\automation-framework-back\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E01E2C-C0C0-4541-8845-5004FC7E4E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBA4CA0-9AE9-49D1-B438-7E77A964C96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
   <si>
     <t>ATC0001_Nueva_Denuncia</t>
   </si>
@@ -168,9 +168,6 @@
     <t>ATC01_Test1</t>
   </si>
   <si>
-    <t>ATC02_Test2</t>
-  </si>
-  <si>
     <t>Id</t>
   </si>
   <si>
@@ -195,10 +192,22 @@
     <t>Ejecutar</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>SI</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>password123</t>
+  </si>
+  <si>
+    <t>ATC02_Booking</t>
   </si>
 </sst>
 </file>
@@ -322,15 +331,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:F3" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:H3" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:H3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
     <tableColumn id="5" xr3:uid="{6BE7C047-30A3-421D-870C-CBBC4443BB44}" name="Ejecutar"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="UserId"/>
     <tableColumn id="3" xr3:uid="{2E8C600E-A409-4D88-8FD4-9D0C9284F1EF}" name="Id_2"/>
     <tableColumn id="6" xr3:uid="{68A333F0-9C06-4364-976F-9304FB37C2B5}" name="Schema"/>
+    <tableColumn id="7" xr3:uid="{7D7EB05F-7DDC-4BE5-8671-AAD24B263E79}" name="Username"/>
+    <tableColumn id="8" xr3:uid="{CCA99CA1-1F34-414C-A772-017976EEB1ED}" name="Password"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -859,19 +870,25 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>49</v>
+      <c r="G1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -879,30 +896,36 @@
         <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
+      <c r="G3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="I6" s="2"/>

</xml_diff>

<commit_message>
feat: New update and delete functionality added
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\eclipse-workspace\automation-framework-back\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBA4CA0-9AE9-49D1-B438-7E77A964C96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E78A6DA-8489-4AF1-A727-E963ABCB4592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="75">
   <si>
     <t>ATC0001_Nueva_Denuncia</t>
   </si>
@@ -208,6 +208,60 @@
   </si>
   <si>
     <t>ATC02_Booking</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>TotalPrice</t>
+  </si>
+  <si>
+    <t>DepositPaid</t>
+  </si>
+  <si>
+    <t>Checkin</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>AdditionalNeeds</t>
+  </si>
+  <si>
+    <t>Osiris</t>
+  </si>
+  <si>
+    <t>Montiel</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Breakfast</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>2025-01-01</t>
+  </si>
+  <si>
+    <t>2025-01-07</t>
+  </si>
+  <si>
+    <t>NewCheckin</t>
+  </si>
+  <si>
+    <t>NewCheckout</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
   </si>
 </sst>
 </file>
@@ -266,7 +320,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -274,6 +328,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -281,13 +336,13 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -306,20 +361,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:P4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TestCaseName"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tester"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Version"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="2"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Descripcion"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Pais"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Subsidiaria"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Categoria"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="FechaInicial"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="1"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="NombrePersona"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="CargoPersona"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="InternoExterno"/>
@@ -331,9 +386,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:H3" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:H3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:Q3" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:Q3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
     <tableColumn id="5" xr3:uid="{6BE7C047-30A3-421D-870C-CBBC4443BB44}" name="Ejecutar"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Id"/>
@@ -342,6 +397,15 @@
     <tableColumn id="6" xr3:uid="{68A333F0-9C06-4364-976F-9304FB37C2B5}" name="Schema"/>
     <tableColumn id="7" xr3:uid="{7D7EB05F-7DDC-4BE5-8671-AAD24B263E79}" name="Username"/>
     <tableColumn id="8" xr3:uid="{CCA99CA1-1F34-414C-A772-017976EEB1ED}" name="Password"/>
+    <tableColumn id="9" xr3:uid="{FB18B245-6FB0-4CB1-8092-4648540361B1}" name="FirstName"/>
+    <tableColumn id="10" xr3:uid="{C2C242FA-2D89-4FD8-9E87-EE52CD560E03}" name="LastName"/>
+    <tableColumn id="11" xr3:uid="{588E9271-E116-4FB4-982B-C5D5FBEB964E}" name="TotalPrice"/>
+    <tableColumn id="12" xr3:uid="{F0351D86-C94F-4F12-8790-1F068C5E787B}" name="DepositPaid"/>
+    <tableColumn id="13" xr3:uid="{A0C08A15-FFB2-42FB-B1B4-598BE02D6B24}" name="Checkin"/>
+    <tableColumn id="14" xr3:uid="{0116807E-E04B-4832-86E0-27D3452C2F54}" name="Checkout"/>
+    <tableColumn id="15" xr3:uid="{D7CE322F-36F3-4557-AA3F-C58076AEB494}" name="AdditionalNeeds"/>
+    <tableColumn id="16" xr3:uid="{9DF1F7F9-C0A6-483E-9C59-9103527B5B93}" name="NewCheckin"/>
+    <tableColumn id="17" xr3:uid="{B9A6880A-F3B4-4C7D-BB9B-7748844E2AF4}" name="NewCheckout"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -854,7 +918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.5546875" bestFit="1" customWidth="1"/>
@@ -863,9 +927,18 @@
     <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -890,8 +963,35 @@
       <c r="H1" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -911,7 +1011,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -926,14 +1026,41 @@
       <c r="H3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J3" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="L3" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="O3" t="s">
+        <v>67</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D8" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enable parallel class execution in TestNG
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\eclipse-workspace\automation-framework-back\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8931575B-EC24-4791-81C0-152A177BB998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A658BBA-A887-4C45-A4F5-F1FE75BBB29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,13 +336,13 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -361,20 +361,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:P4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TestCaseName"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tester"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Version"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Descripcion"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Pais"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Subsidiaria"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Categoria"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="FechaInicial"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="0"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="NombrePersona"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="CargoPersona"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="InternoExterno"/>
@@ -386,7 +386,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:Q3" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:Q3" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:Q3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
@@ -918,7 +918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.5546875" bestFit="1" customWidth="1"/>
@@ -1054,15 +1054,6 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D8" s="2"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>